<commit_message>
Seller order sheets take every cell style from a blank copy of the team's purchase form
</commit_message>
<xml_diff>
--- a/docs/vendor-orders/adafruit.xlsx
+++ b/docs/vendor-orders/adafruit.xlsx
@@ -16,10 +16,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="1">
+  <numFmts count="2">
     <numFmt numFmtId="164" formatCode="_(&quot;$&quot;* #,##0.00_);_(&quot;$&quot;* \(#,##0.00\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
+    <numFmt numFmtId="165" formatCode="_([$$-409]* #,##0.00_);_([$$-409]* \(#,##0.00\);_([$$-409]* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="8">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -28,7 +29,42 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Arial"/>
+      <color rgb="FF333333"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color rgb="FF000000"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <color rgb="FF0000FF"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FFFF0000"/>
+      <sz val="11"/>
+      <u val="single"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <color theme="1"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="FF000000"/>
+      <sz val="11"/>
     </font>
   </fonts>
   <fills count="3">
@@ -41,10 +77,11 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF4B083"/>
+        <bgColor rgb="FFF4B083"/>
       </patternFill>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -52,16 +89,50 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom/>
+    </border>
+    <border/>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="14">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="164" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="1" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="164" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
+    <xf numFmtId="165" fontId="2" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="164" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="6" fillId="0" borderId="2" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="164" fontId="7" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -430,43 +501,43 @@
   <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="45" customWidth="1" min="1" max="1"/>
+    <col width="39.57" customWidth="1" min="1" max="1"/>
     <col width="9" customWidth="1" min="2" max="2"/>
     <col width="14.29" customWidth="1" min="3" max="3"/>
     <col width="11" customWidth="1" min="4" max="4"/>
     <col width="28" customWidth="1" min="5" max="5"/>
-    <col width="60" customWidth="1" min="6" max="6"/>
     <col width="86.29000000000001" customWidth="1" min="7" max="7"/>
     <col width="11" customWidth="1" min="8" max="8"/>
+    <col width="8.710000000000001" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="32.25" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Item</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>Quantity</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="3" t="inlineStr">
         <is>
           <t>Cost per Item</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="3" t="inlineStr">
         <is>
           <t>Total Cost</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="3" t="inlineStr">
         <is>
           <t>Item/SKU Number</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="3" t="inlineStr">
         <is>
           <t xml:space="preserve">Other Specs if Applicable </t>
         </is>
@@ -476,65 +547,65 @@
           <t>Link</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="3" t="inlineStr">
         <is>
           <t>Total</t>
         </is>
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="inlineStr">
+      <c r="A2" s="4" t="inlineStr">
         <is>
           <t>Adafruit LIS3MDL magnetometer breakout (product 4479)</t>
         </is>
       </c>
-      <c r="B2" t="n">
+      <c r="B2" s="5" t="n">
         <v>1</v>
       </c>
-      <c r="C2" s="2" t="n">
+      <c r="C2" s="6" t="n">
         <v>9.949999999999999</v>
       </c>
-      <c r="D2" s="2">
+      <c r="D2" s="7">
         <f>B2*C2</f>
         <v/>
       </c>
-      <c r="E2" t="inlineStr">
+      <c r="E2" s="4" t="inlineStr">
         <is>
           <t>Adafruit LIS3MDL magnetometer breakout (product 4479)</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr">
+      <c r="F2" s="4" t="inlineStr">
         <is>
           <t>Drone; Compass, 1.5 g; Shares the I2C wires of the J5 or J8 cable. Runs from that cable's 5 V.</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr">
+      <c r="G2" s="8" t="inlineStr">
         <is>
           <t>https://www.adafruit.com/product/4479</t>
         </is>
       </c>
-      <c r="H2" s="2">
+      <c r="H2" s="9">
         <f>D2</f>
         <v/>
       </c>
     </row>
     <row r="3">
-      <c r="G3" s="3" t="inlineStr">
+      <c r="G3" s="10" t="inlineStr">
         <is>
           <t>Please select fastest shipping available</t>
         </is>
       </c>
-      <c r="H3" s="2" t="n">
+      <c r="H3" s="11" t="n">
         <v>0</v>
       </c>
     </row>
     <row r="4">
-      <c r="G4" s="3" t="inlineStr">
+      <c r="G4" s="12" t="inlineStr">
         <is>
           <t>Grand Total</t>
         </is>
       </c>
-      <c r="H4" s="4">
+      <c r="H4" s="13">
         <f>SUM(H2:H3)</f>
         <v/>
       </c>

</xml_diff>